<commit_message>
feat: year-end settlement, RTE tracking, promotion & roll number fixes
- Year-end settlement now includes RTE students (mode='all') so govt fees can be formally tracked and settled
- Added Category badge column to year-end settlement table
- RTE report gains Due/Received/Pending/Status columns per student
- Defaulters report: replaced toggle with Parent/RTE mode switch, removed Avg Balance card, fixed custom fee due calculation
- Roll numbers reassigned by admission date (confirmed_date) not name
- Promotion page: renamed column to General ID / DGA No, pre-fills from student record
- Admission show: displays both DGA and General ID badges; warns when General ID missing for Class 1+
- Removed duplicate Reassign Roll Numbers button from promotions index (lives in Academic Settings)
- Updated import files: 11 defaulters with partial/zero payment, rest fully paid

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/schoolDocs/StudentImportData/Class1_ImportReady.xlsx
+++ b/schoolDocs/StudentImportData/Class1_ImportReady.xlsx
@@ -709,27 +709,27 @@
   <dimension ref="A1:U20"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="9.283" bestFit="true" customWidth="true" style="0"/>
-    <col min="2" max="2" width="37.705" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="18.71" bestFit="true" customWidth="true" style="0"/>
-    <col min="4" max="4" width="10.426" bestFit="true" customWidth="true" style="0"/>
-    <col min="5" max="5" width="9.283" bestFit="true" customWidth="true" style="0"/>
-    <col min="6" max="6" width="11.569" bestFit="true" customWidth="true" style="0"/>
-    <col min="7" max="7" width="25.708" bestFit="true" customWidth="true" style="0"/>
-    <col min="8" max="8" width="17.567" bestFit="true" customWidth="true" style="0"/>
-    <col min="9" max="9" width="15.139" bestFit="true" customWidth="true" style="0"/>
-    <col min="10" max="10" width="24.565" bestFit="true" customWidth="true" style="0"/>
-    <col min="11" max="11" width="29.279" bestFit="true" customWidth="true" style="0"/>
-    <col min="12" max="12" width="35.277" bestFit="true" customWidth="true" style="0"/>
-    <col min="13" max="13" width="13.997" bestFit="true" customWidth="true" style="0"/>
-    <col min="14" max="14" width="26.993" bestFit="true" customWidth="true" style="0"/>
-    <col min="15" max="15" width="16.282" bestFit="true" customWidth="true" style="0"/>
-    <col min="16" max="16" width="31.707" bestFit="true" customWidth="true" style="0"/>
-    <col min="17" max="17" width="16.282" bestFit="true" customWidth="true" style="0"/>
-    <col min="18" max="18" width="25.851" bestFit="true" customWidth="true" style="0"/>
-    <col min="19" max="19" width="15.139" bestFit="true" customWidth="true" style="0"/>
-    <col min="20" max="20" width="22.28" bestFit="true" customWidth="true" style="0"/>
-    <col min="21" max="21" width="108.402" bestFit="true" customWidth="true" style="0"/>
+    <col min="1" max="1" width="9.283" customWidth="true" style="0"/>
+    <col min="2" max="2" width="37.705" customWidth="true" style="0"/>
+    <col min="3" max="3" width="18.71" customWidth="true" style="0"/>
+    <col min="4" max="4" width="10.426" customWidth="true" style="0"/>
+    <col min="5" max="5" width="9.283" customWidth="true" style="0"/>
+    <col min="6" max="6" width="11.569" customWidth="true" style="0"/>
+    <col min="7" max="7" width="25.708" customWidth="true" style="0"/>
+    <col min="8" max="8" width="17.567" customWidth="true" style="0"/>
+    <col min="9" max="9" width="15.139" customWidth="true" style="0"/>
+    <col min="10" max="10" width="24.565" customWidth="true" style="0"/>
+    <col min="11" max="11" width="29.279" customWidth="true" style="0"/>
+    <col min="12" max="12" width="35.277" customWidth="true" style="0"/>
+    <col min="13" max="13" width="13.997" customWidth="true" style="0"/>
+    <col min="14" max="14" width="26.993" customWidth="true" style="0"/>
+    <col min="15" max="15" width="16.282" customWidth="true" style="0"/>
+    <col min="16" max="16" width="31.707" customWidth="true" style="0"/>
+    <col min="17" max="17" width="16.282" customWidth="true" style="0"/>
+    <col min="18" max="18" width="25.851" customWidth="true" style="0"/>
+    <col min="19" max="19" width="15.139" customWidth="true" style="0"/>
+    <col min="20" max="20" width="22.28" customWidth="true" style="0"/>
+    <col min="21" max="21" width="108.402" customWidth="true" style="0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:21" customHeight="1" ht="30">
@@ -819,6 +819,11 @@
       <c r="H2" t="s">
         <v>25</v>
       </c>
+      <c r="I2"/>
+      <c r="J2"/>
+      <c r="K2">
+        <v>0</v>
+      </c>
       <c r="L2" t="s">
         <v>26</v>
       </c>
@@ -860,6 +865,11 @@
       <c r="H3" t="s">
         <v>25</v>
       </c>
+      <c r="I3"/>
+      <c r="J3"/>
+      <c r="K3">
+        <v>0</v>
+      </c>
       <c r="L3" t="s">
         <v>33</v>
       </c>
@@ -901,6 +911,8 @@
       <c r="H4" t="s">
         <v>38</v>
       </c>
+      <c r="I4"/>
+      <c r="J4"/>
       <c r="K4">
         <v>16200</v>
       </c>
@@ -936,6 +948,11 @@
       <c r="H5" t="s">
         <v>25</v>
       </c>
+      <c r="I5"/>
+      <c r="J5"/>
+      <c r="K5">
+        <v>0</v>
+      </c>
       <c r="L5" t="s">
         <v>42</v>
       </c>
@@ -977,6 +994,8 @@
       <c r="H6" t="s">
         <v>38</v>
       </c>
+      <c r="I6"/>
+      <c r="J6"/>
       <c r="K6">
         <v>16200</v>
       </c>
@@ -1018,8 +1037,10 @@
       <c r="H7" t="s">
         <v>38</v>
       </c>
+      <c r="I7"/>
+      <c r="J7"/>
       <c r="K7">
-        <v>16200</v>
+        <v>0</v>
       </c>
       <c r="L7" t="s">
         <v>51</v>
@@ -1059,6 +1080,7 @@
       <c r="I8">
         <v>50</v>
       </c>
+      <c r="J8"/>
       <c r="K8">
         <v>8100</v>
       </c>
@@ -1100,8 +1122,10 @@
       <c r="H9" t="s">
         <v>61</v>
       </c>
+      <c r="I9"/>
+      <c r="J9"/>
       <c r="K9">
-        <v>12200</v>
+        <v>16200</v>
       </c>
       <c r="L9" t="s">
         <v>62</v>
@@ -1141,8 +1165,9 @@
       <c r="I10">
         <v>75</v>
       </c>
+      <c r="J10"/>
       <c r="K10" s="5">
-        <v>2000</v>
+        <v>4050</v>
       </c>
       <c r="L10" t="s">
         <v>67</v>
@@ -1176,6 +1201,8 @@
       <c r="H11" t="s">
         <v>61</v>
       </c>
+      <c r="I11"/>
+      <c r="J11"/>
       <c r="K11">
         <v>16200</v>
       </c>
@@ -1214,8 +1241,10 @@
       <c r="H12" t="s">
         <v>38</v>
       </c>
+      <c r="I12"/>
+      <c r="J12"/>
       <c r="K12" s="5">
-        <v>7000</v>
+        <v>16200</v>
       </c>
       <c r="L12" t="s">
         <v>73</v>
@@ -1249,6 +1278,8 @@
       <c r="H13" t="s">
         <v>61</v>
       </c>
+      <c r="I13"/>
+      <c r="J13"/>
       <c r="K13">
         <v>16200</v>
       </c>
@@ -1287,6 +1318,11 @@
       <c r="H14" t="s">
         <v>25</v>
       </c>
+      <c r="I14"/>
+      <c r="J14"/>
+      <c r="K14">
+        <v>0</v>
+      </c>
       <c r="L14" t="s">
         <v>78</v>
       </c>
@@ -1319,8 +1355,10 @@
       <c r="H15" t="s">
         <v>38</v>
       </c>
+      <c r="I15"/>
+      <c r="J15"/>
       <c r="K15" s="5">
-        <v>9450</v>
+        <v>16200</v>
       </c>
       <c r="L15" t="s">
         <v>80</v>
@@ -1357,8 +1395,10 @@
       <c r="H16" t="s">
         <v>38</v>
       </c>
+      <c r="I16"/>
+      <c r="J16"/>
       <c r="K16" s="5">
-        <v>5000</v>
+        <v>12200</v>
       </c>
       <c r="L16" t="s">
         <v>84</v>
@@ -1398,6 +1438,11 @@
       <c r="H17" t="s">
         <v>25</v>
       </c>
+      <c r="I17"/>
+      <c r="J17"/>
+      <c r="K17">
+        <v>0</v>
+      </c>
       <c r="L17" t="s">
         <v>87</v>
       </c>
@@ -1436,6 +1481,10 @@
       <c r="I18">
         <v>25</v>
       </c>
+      <c r="J18"/>
+      <c r="K18">
+        <v>9150</v>
+      </c>
       <c r="L18" t="s">
         <v>89</v>
       </c>
@@ -1477,6 +1526,8 @@
       <c r="H19" t="s">
         <v>38</v>
       </c>
+      <c r="I19"/>
+      <c r="J19"/>
       <c r="K19">
         <v>12200</v>
       </c>
@@ -1511,6 +1562,11 @@
       </c>
       <c r="H20" t="s">
         <v>25</v>
+      </c>
+      <c r="I20"/>
+      <c r="J20"/>
+      <c r="K20">
+        <v>0</v>
       </c>
       <c r="L20" t="s">
         <v>51</v>

</xml_diff>

<commit_message>
feat: add rte_application_no to import pipeline and update all import files
- Column U added to import template and all 11 xlsx files: RTE Application No
- Import validates: alphanumeric max 20 chars, only allowed when fee_category = rte
- AdmissionRepository create() saves rte_application_no (uppercase) on import
- All 11 xlsx files: cleared old stale notes from column U, backfilled dummy RTE numbers (25MSxxxxxx) for all 53 RTE students from local DB
- General ID column (S) left blank — Class 1-8 IDs to be filled with real ZP numbers before staging import

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/schoolDocs/StudentImportData/Class1_ImportReady.xlsx
+++ b/schoolDocs/StudentImportData/Class1_ImportReady.xlsx
@@ -14,8 +14,34 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Author</author>
+  </authors>
+  <commentList>
+    <comment ref="U1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <rFont val="Calibri"/>
+            <b val="false"/>
+            <i val="false"/>
+            <strike val="false"/>
+            <color rgb="FF000000"/>
+            <sz val="11"/>
+            <u val="none"/>
+          </rPr>
+          <t xml:space="preserve">Only for RTE students. Alphanumeric, e.g. 26MS011157 (Year+StateCode+Sequence). Leave blank for non-RTE.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="96">
   <si>
     <t>Sr No</t>
   </si>
@@ -77,7 +103,7 @@
     <t>DGA Admission No</t>
   </si>
   <si>
-    <t>Notes for Verification (ignored on import)</t>
+    <t>RTE Application No</t>
   </si>
   <si>
     <t>Pranav Sharad Gorgal</t>
@@ -110,7 +136,7 @@
     <t>Home Maker</t>
   </si>
   <si>
-    <t>RTE — fees paid by government</t>
+    <t>25MS000006</t>
   </si>
   <si>
     <t>Om Sunil Ingle</t>
@@ -128,6 +154,9 @@
     <t>Work in Company</t>
   </si>
   <si>
+    <t>25MS000007</t>
+  </si>
+  <si>
     <t>Devansh Swapnil Jadhav</t>
   </si>
   <si>
@@ -158,6 +187,9 @@
     <t>Works at her own farm</t>
   </si>
   <si>
+    <t>25MS000008</t>
+  </si>
+  <si>
     <t>Kartik D Nevase</t>
   </si>
   <si>
@@ -194,9 +226,6 @@
     <t>Bakery shop on wheelbarrow</t>
   </si>
   <si>
-    <t>Discount 50% on boys fee ₹16200 = ₹8100 payable — full paid</t>
-  </si>
-  <si>
     <t>Ayush Asgar Shaikh</t>
   </si>
   <si>
@@ -212,36 +241,24 @@
     <t>19km</t>
   </si>
   <si>
-    <t>DGA shows ₹12200 for this CoC boy — system will use ₹16200. Please verify.</t>
-  </si>
-  <si>
     <t>Samarthraj Ajithkumar Desinayak</t>
   </si>
   <si>
     <t>15/01/2025</t>
   </si>
   <si>
-    <t>75% discount on boys ₹16200 = ₹4050 payable — collected ₹2000 (partial). Verify discount %.</t>
-  </si>
-  <si>
     <t>Jivnath Navnath Pawar</t>
   </si>
   <si>
     <t>18/12/2022</t>
   </si>
   <si>
-    <t>CoC student — full ₹16200 collected</t>
-  </si>
-  <si>
     <t>Vedansh Popat Yale</t>
   </si>
   <si>
     <t>31/01/2025</t>
   </si>
   <si>
-    <t>Partial — ₹7000 of ₹16200 collected</t>
-  </si>
-  <si>
     <t>Swaraj Lakshman Kashid</t>
   </si>
   <si>
@@ -254,15 +271,15 @@
     <t>07/01/2023</t>
   </si>
   <si>
+    <t>25MS000009</t>
+  </si>
+  <si>
     <t>Aryan Ganesh Pawar</t>
   </si>
   <si>
     <t>22/12/2022</t>
   </si>
   <si>
-    <t>Partial — ₹9450 of ₹16200 collected</t>
-  </si>
-  <si>
     <t>Chaitrali Rahul Chaudhari</t>
   </si>
   <si>
@@ -272,15 +289,15 @@
     <t>07/01/2025</t>
   </si>
   <si>
-    <t>Partial — ₹5000 of ₹12200 collected</t>
-  </si>
-  <si>
     <t>Shravani Amit Kale</t>
   </si>
   <si>
     <t>08/02/2025</t>
   </si>
   <si>
+    <t>25MS000010</t>
+  </si>
+  <si>
     <t>Divya Dada Kokre</t>
   </si>
   <si>
@@ -290,9 +307,6 @@
     <t>Shepherd</t>
   </si>
   <si>
-    <t>Discount 25% on girls fee ₹12200 = ₹9150 payable — collected ₹0</t>
-  </si>
-  <si>
     <t>Blessing Deepak Tujare</t>
   </si>
   <si>
@@ -312,6 +326,9 @@
   </si>
   <si>
     <t>Tasty Bites Company</t>
+  </si>
+  <si>
+    <t>25MS000011</t>
   </si>
 </sst>
 </file>
@@ -363,12 +380,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF7B3F00"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFFF3CD"/>
         <bgColor rgb="FF000000"/>
       </patternFill>
@@ -376,6 +387,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD5EAD0"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2E4057"/>
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
@@ -397,16 +414,16 @@
     <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="3" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="3" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="2" numFmtId="0" fillId="4" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="2" numFmtId="0" fillId="5" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="3" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="5" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="4" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -729,7 +746,7 @@
     <col min="18" max="18" width="25.851" customWidth="true" style="0"/>
     <col min="19" max="19" width="15.139" customWidth="true" style="0"/>
     <col min="20" max="20" width="22.28" customWidth="true" style="0"/>
-    <col min="21" max="21" width="108.402" customWidth="true" style="0"/>
+    <col min="21" max="21" width="20" customWidth="true" style="0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:21" customHeight="1" ht="30">
@@ -763,10 +780,10 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="3" t="s">
         <v>11</v>
       </c>
       <c r="M1" s="1" t="s">
@@ -793,7 +810,7 @@
       <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="U1" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -886,7 +903,7 @@
         <v>30</v>
       </c>
       <c r="U3" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:21">
@@ -894,7 +911,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D4" t="s">
         <v>22</v>
@@ -909,7 +926,7 @@
         <v>9767689897</v>
       </c>
       <c r="H4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I4"/>
       <c r="J4"/>
@@ -917,21 +934,22 @@
         <v>16200</v>
       </c>
       <c r="L4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="M4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="N4" t="s">
         <v>28</v>
       </c>
+      <c r="U4"/>
     </row>
     <row r="5" spans="1:21">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D5" t="s">
         <v>22</v>
@@ -954,22 +972,22 @@
         <v>0</v>
       </c>
       <c r="L5" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="M5" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="N5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="P5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="R5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="U5" t="s">
-        <v>31</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:21">
@@ -977,7 +995,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D6" t="s">
         <v>22</v>
@@ -992,7 +1010,7 @@
         <v>8677867777</v>
       </c>
       <c r="H6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I6"/>
       <c r="J6"/>
@@ -1000,27 +1018,28 @@
         <v>16200</v>
       </c>
       <c r="L6" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="M6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="N6" t="s">
         <v>28</v>
       </c>
       <c r="P6" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="R6" t="s">
         <v>30</v>
       </c>
+      <c r="U6"/>
     </row>
     <row r="7" spans="1:21">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D7" t="s">
         <v>22</v>
@@ -1035,7 +1054,7 @@
         <v>9370401366</v>
       </c>
       <c r="H7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I7"/>
       <c r="J7"/>
@@ -1043,7 +1062,7 @@
         <v>0</v>
       </c>
       <c r="L7" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="M7" t="s">
         <v>34</v>
@@ -1052,15 +1071,16 @@
         <v>35</v>
       </c>
       <c r="P7" t="s">
-        <v>52</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="U7"/>
     </row>
     <row r="8" spans="1:21">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D8" t="s">
         <v>22</v>
@@ -1075,7 +1095,7 @@
         <v>6395064076</v>
       </c>
       <c r="H8" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I8">
         <v>50</v>
@@ -1085,30 +1105,28 @@
         <v>8100</v>
       </c>
       <c r="L8" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="M8" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="N8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="P8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="R8" t="s">
         <v>30</v>
       </c>
-      <c r="U8" t="s">
-        <v>59</v>
-      </c>
+      <c r="U8"/>
     </row>
     <row r="9" spans="1:21">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D9" t="s">
         <v>22</v>
@@ -1120,7 +1138,7 @@
         <v>24</v>
       </c>
       <c r="H9" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="I9"/>
       <c r="J9"/>
@@ -1128,17 +1146,15 @@
         <v>16200</v>
       </c>
       <c r="L9" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="M9" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="N9" t="s">
-        <v>64</v>
-      </c>
-      <c r="U9" s="5" t="s">
         <v>65</v>
       </c>
+      <c r="U9" s="4"/>
     </row>
     <row r="10" spans="1:21">
       <c r="A10">
@@ -1160,13 +1176,13 @@
         <v>7720870317</v>
       </c>
       <c r="H10" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I10">
         <v>75</v>
       </c>
       <c r="J10"/>
-      <c r="K10" s="5">
+      <c r="K10" s="4">
         <v>4050</v>
       </c>
       <c r="L10" t="s">
@@ -1176,18 +1192,16 @@
         <v>27</v>
       </c>
       <c r="N10" t="s">
-        <v>64</v>
-      </c>
-      <c r="U10" s="5" t="s">
-        <v>68</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="U10" s="4"/>
     </row>
     <row r="11" spans="1:21">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D11" t="s">
         <v>22</v>
@@ -1199,7 +1213,7 @@
         <v>24</v>
       </c>
       <c r="H11" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="I11"/>
       <c r="J11"/>
@@ -1207,24 +1221,22 @@
         <v>16200</v>
       </c>
       <c r="L11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="M11" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="N11" t="s">
-        <v>64</v>
-      </c>
-      <c r="U11" t="s">
-        <v>71</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="U11"/>
     </row>
     <row r="12" spans="1:21">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D12" t="s">
         <v>22</v>
@@ -1239,15 +1251,15 @@
         <v>9975609853</v>
       </c>
       <c r="H12" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I12"/>
       <c r="J12"/>
-      <c r="K12" s="5">
+      <c r="K12" s="4">
         <v>16200</v>
       </c>
       <c r="L12" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="M12" t="s">
         <v>27</v>
@@ -1255,16 +1267,14 @@
       <c r="N12" t="s">
         <v>28</v>
       </c>
-      <c r="U12" t="s">
-        <v>74</v>
-      </c>
+      <c r="U12"/>
     </row>
     <row r="13" spans="1:21">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D13" t="s">
         <v>22</v>
@@ -1276,7 +1286,7 @@
         <v>24</v>
       </c>
       <c r="H13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="I13"/>
       <c r="J13"/>
@@ -1284,24 +1294,22 @@
         <v>16200</v>
       </c>
       <c r="L13" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="M13" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="N13" t="s">
-        <v>64</v>
-      </c>
-      <c r="U13" t="s">
-        <v>71</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="U13"/>
     </row>
     <row r="14" spans="1:21">
       <c r="A14">
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D14" t="s">
         <v>22</v>
@@ -1324,16 +1332,16 @@
         <v>0</v>
       </c>
       <c r="L14" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="M14" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="N14" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="U14" t="s">
-        <v>31</v>
+        <v>76</v>
       </c>
     </row>
     <row r="15" spans="1:21">
@@ -1341,7 +1349,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D15" t="s">
         <v>22</v>
@@ -1353,35 +1361,33 @@
         <v>24</v>
       </c>
       <c r="H15" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I15"/>
       <c r="J15"/>
-      <c r="K15" s="5">
+      <c r="K15" s="4">
         <v>16200</v>
       </c>
       <c r="L15" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="M15" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="N15" t="s">
-        <v>57</v>
-      </c>
-      <c r="U15" t="s">
-        <v>81</v>
-      </c>
+        <v>59</v>
+      </c>
+      <c r="U15"/>
     </row>
     <row r="16" spans="1:21">
       <c r="A16">
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="D16" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E16" t="s">
         <v>23</v>
@@ -1393,15 +1399,15 @@
         <v>9923355136</v>
       </c>
       <c r="H16" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I16"/>
       <c r="J16"/>
-      <c r="K16" s="5">
+      <c r="K16" s="4">
         <v>12200</v>
       </c>
       <c r="L16" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="M16" t="s">
         <v>34</v>
@@ -1410,21 +1416,19 @@
         <v>35</v>
       </c>
       <c r="P16" t="s">
-        <v>52</v>
-      </c>
-      <c r="U16" t="s">
-        <v>85</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="U16"/>
     </row>
     <row r="17" spans="1:21">
       <c r="A17">
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="D17" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E17" t="s">
         <v>23</v>
@@ -1444,16 +1448,16 @@
         <v>0</v>
       </c>
       <c r="L17" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="M17" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="N17" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="U17" t="s">
-        <v>31</v>
+        <v>84</v>
       </c>
     </row>
     <row r="18" spans="1:21">
@@ -1461,10 +1465,10 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="D18" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E18" t="s">
         <v>23</v>
@@ -1476,7 +1480,7 @@
         <v>9834614015</v>
       </c>
       <c r="H18" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I18">
         <v>25</v>
@@ -1486,33 +1490,31 @@
         <v>9150</v>
       </c>
       <c r="L18" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="M18" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="N18" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="P18" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="R18" t="s">
         <v>30</v>
       </c>
-      <c r="U18" t="s">
-        <v>91</v>
-      </c>
+      <c r="U18"/>
     </row>
     <row r="19" spans="1:21">
       <c r="A19">
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="D19" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E19" t="s">
         <v>23</v>
@@ -1524,7 +1526,7 @@
         <v>9529295079</v>
       </c>
       <c r="H19" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I19"/>
       <c r="J19"/>
@@ -1532,24 +1534,25 @@
         <v>12200</v>
       </c>
       <c r="L19" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="M19" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="N19" t="s">
-        <v>95</v>
-      </c>
+        <v>91</v>
+      </c>
+      <c r="U19"/>
     </row>
     <row r="20" spans="1:21">
       <c r="A20">
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D20" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E20" t="s">
         <v>23</v>
@@ -1569,22 +1572,22 @@
         <v>0</v>
       </c>
       <c r="L20" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="M20" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="N20" t="s">
         <v>28</v>
       </c>
       <c r="P20" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="R20" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="U20" t="s">
-        <v>31</v>
+        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -1599,6 +1602,7 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
+  <legacyDrawing r:id="rId_comments_vml1"/>
   <tableParts count="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: backfill General IDs into Class 1-8 import files
All Class 1-8 xlsx files now have dummy 27-prefix General IDs in column S,
matching what was inserted directly into the local DB. Import files now contain
all three DB-direct fields: admission date (L), General ID (S), RTE App No (U).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/schoolDocs/StudentImportData/Class1_ImportReady.xlsx
+++ b/schoolDocs/StudentImportData/Class1_ImportReady.xlsx
@@ -856,6 +856,9 @@
       <c r="R2" t="s">
         <v>30</v>
       </c>
+      <c r="S2">
+        <v>27000010001</v>
+      </c>
       <c r="U2" t="s">
         <v>31</v>
       </c>
@@ -902,6 +905,9 @@
       <c r="R3" t="s">
         <v>30</v>
       </c>
+      <c r="S3">
+        <v>27000010002</v>
+      </c>
       <c r="U3" t="s">
         <v>37</v>
       </c>
@@ -942,6 +948,9 @@
       <c r="N4" t="s">
         <v>28</v>
       </c>
+      <c r="S4">
+        <v>27000010003</v>
+      </c>
       <c r="U4"/>
     </row>
     <row r="5" spans="1:21">
@@ -986,6 +995,9 @@
       <c r="R5" t="s">
         <v>47</v>
       </c>
+      <c r="S5">
+        <v>27000010004</v>
+      </c>
       <c r="U5" t="s">
         <v>48</v>
       </c>
@@ -1032,6 +1044,9 @@
       <c r="R6" t="s">
         <v>30</v>
       </c>
+      <c r="S6">
+        <v>27000010005</v>
+      </c>
       <c r="U6"/>
     </row>
     <row r="7" spans="1:21">
@@ -1073,6 +1088,9 @@
       <c r="P7" t="s">
         <v>54</v>
       </c>
+      <c r="S7">
+        <v>27000010006</v>
+      </c>
       <c r="U7"/>
     </row>
     <row r="8" spans="1:21">
@@ -1118,6 +1136,9 @@
       </c>
       <c r="R8" t="s">
         <v>30</v>
+      </c>
+      <c r="S8">
+        <v>27000010007</v>
       </c>
       <c r="U8"/>
     </row>
@@ -1154,6 +1175,9 @@
       <c r="N9" t="s">
         <v>65</v>
       </c>
+      <c r="S9">
+        <v>27000010008</v>
+      </c>
       <c r="U9" s="4"/>
     </row>
     <row r="10" spans="1:21">
@@ -1193,6 +1217,9 @@
       </c>
       <c r="N10" t="s">
         <v>65</v>
+      </c>
+      <c r="S10">
+        <v>27000010009</v>
       </c>
       <c r="U10" s="4"/>
     </row>
@@ -1229,6 +1256,9 @@
       <c r="N11" t="s">
         <v>65</v>
       </c>
+      <c r="S11">
+        <v>27000010010</v>
+      </c>
       <c r="U11"/>
     </row>
     <row r="12" spans="1:21">
@@ -1267,6 +1297,9 @@
       <c r="N12" t="s">
         <v>28</v>
       </c>
+      <c r="S12">
+        <v>27000010011</v>
+      </c>
       <c r="U12"/>
     </row>
     <row r="13" spans="1:21">
@@ -1302,6 +1335,9 @@
       <c r="N13" t="s">
         <v>65</v>
       </c>
+      <c r="S13">
+        <v>27000010012</v>
+      </c>
       <c r="U13"/>
     </row>
     <row r="14" spans="1:21">
@@ -1340,6 +1376,9 @@
       <c r="N14" t="s">
         <v>59</v>
       </c>
+      <c r="S14">
+        <v>27000010013</v>
+      </c>
       <c r="U14" t="s">
         <v>76</v>
       </c>
@@ -1377,6 +1416,9 @@
       <c r="N15" t="s">
         <v>59</v>
       </c>
+      <c r="S15">
+        <v>27000010014</v>
+      </c>
       <c r="U15"/>
     </row>
     <row r="16" spans="1:21">
@@ -1418,6 +1460,9 @@
       <c r="P16" t="s">
         <v>54</v>
       </c>
+      <c r="S16">
+        <v>27000010015</v>
+      </c>
       <c r="U16"/>
     </row>
     <row r="17" spans="1:21">
@@ -1456,6 +1501,9 @@
       <c r="N17" t="s">
         <v>59</v>
       </c>
+      <c r="S17">
+        <v>27000010016</v>
+      </c>
       <c r="U17" t="s">
         <v>84</v>
       </c>
@@ -1503,6 +1551,9 @@
       </c>
       <c r="R18" t="s">
         <v>30</v>
+      </c>
+      <c r="S18">
+        <v>27000010017</v>
       </c>
       <c r="U18"/>
     </row>
@@ -1542,6 +1593,9 @@
       <c r="N19" t="s">
         <v>91</v>
       </c>
+      <c r="S19">
+        <v>27000010018</v>
+      </c>
       <c r="U19"/>
     </row>
     <row r="20" spans="1:21">
@@ -1585,6 +1639,9 @@
       </c>
       <c r="R20" t="s">
         <v>94</v>
+      </c>
+      <c r="S20">
+        <v>27000010019</v>
       </c>
       <c r="U20" t="s">
         <v>95</v>

</xml_diff>